<commit_message>
data: update BuxWV, RCT
</commit_message>
<xml_diff>
--- a/xlsx/RCT.xlsx
+++ b/xlsx/RCT.xlsx
@@ -9,13 +9,13 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="21942" windowHeight="9805"/>
+    <workbookView windowWidth="21942" windowHeight="9600"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$71</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="179">
   <si>
     <t>SORT</t>
   </si>
@@ -58,9 +58,6 @@
     <t>Note</t>
   </si>
   <si>
-    <t>Rec_rcmd</t>
-  </si>
-  <si>
     <t>RCT 1</t>
   </si>
   <si>
@@ -73,6 +70,9 @@
     <t>A minor</t>
   </si>
   <si>
+    <t>Harpsichord</t>
+  </si>
+  <si>
     <t>RCT 2</t>
   </si>
   <si>
@@ -130,7 +130,7 @@
     <t>RCT 7</t>
   </si>
   <si>
-    <t>Premier concert</t>
+    <t>Premier Concert</t>
   </si>
   <si>
     <t>Pièces de clavecin en concerts #1</t>
@@ -139,7 +139,7 @@
     <t>RCT 8</t>
   </si>
   <si>
-    <t>Deuxième concert</t>
+    <t>Deuxième Concert</t>
   </si>
   <si>
     <t>Pièces de clavecin en concerts #2</t>
@@ -157,7 +157,7 @@
     <t>RCT 10</t>
   </si>
   <si>
-    <t>Quatrième concert</t>
+    <t>Quatrième Concert</t>
   </si>
   <si>
     <t>B-flat major</t>
@@ -169,7 +169,7 @@
     <t>RCT 11</t>
   </si>
   <si>
-    <t>Cinquième concert</t>
+    <t>Cinquième Concert</t>
   </si>
   <si>
     <t>Pièces de clavecin en concerts #5</t>
@@ -229,6 +229,18 @@
     <t>Ah! loin de rire, pleurons</t>
   </si>
   <si>
+    <t>RCT 18</t>
+  </si>
+  <si>
+    <t>Avec du vin, endormons-nous, Canon à la 4te</t>
+  </si>
+  <si>
+    <t>Canon</t>
+  </si>
+  <si>
+    <t>E major</t>
+  </si>
+  <si>
     <t>RCT 18bis</t>
   </si>
   <si>
@@ -238,15 +250,6 @@
     <t>formerly attributed to François Couperin</t>
   </si>
   <si>
-    <t>RCT 18</t>
-  </si>
-  <si>
-    <t>Avec du vin, endormons-nous, Canon à la 4te</t>
-  </si>
-  <si>
-    <t>E major</t>
-  </si>
-  <si>
     <t>RCT 19</t>
   </si>
   <si>
@@ -259,7 +262,7 @@
     <t>Réveillez-vous, dormeur sans fin</t>
   </si>
   <si>
-    <t>RCT 2obis</t>
+    <t>RCT 20bis</t>
   </si>
   <si>
     <t>Si tu ne prends garde à toi</t>
@@ -316,6 +319,9 @@
     <t>[Cantate pour le jour de la Saint-Louïs]</t>
   </si>
   <si>
+    <t>Cantata</t>
+  </si>
+  <si>
     <t>RCT 26</t>
   </si>
   <si>
@@ -500,9 +506,6 @@
   </si>
   <si>
     <t>Platée, ou Junon jalouse</t>
-  </si>
-  <si>
-    <t>https://open.spotify.com/album/0AKlp3UyebGKt4o0GShbdg</t>
   </si>
   <si>
     <t>RCT 54</t>
@@ -1197,7 +1200,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1215,9 +1218,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1744,20 +1744,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H71"/>
-  <sheetFormatPr defaultColWidth="8.61261261261261" defaultRowHeight="20" customHeight="1" outlineLevelCol="7"/>
+  <dimension ref="A1:G71"/>
+  <sheetFormatPr defaultColWidth="8.61261261261261" defaultRowHeight="20" customHeight="1" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="6.63963963963964" style="2" customWidth="1"/>
     <col min="2" max="2" width="10.4144144144144" style="2" customWidth="1"/>
-    <col min="3" max="3" width="56.0720720720721" style="3" customWidth="1"/>
+    <col min="3" max="3" width="42.1531531531532" style="3" customWidth="1"/>
     <col min="4" max="4" width="20.1171171171171" style="2" customWidth="1"/>
-    <col min="5" max="5" width="9.18018018018018" style="2" customWidth="1"/>
-    <col min="6" max="7" width="14.0540540540541" style="3" customWidth="1"/>
-    <col min="8" max="8" width="10.5675675675676" style="4" customWidth="1"/>
-    <col min="9" max="16384" width="8.61261261261261" style="4"/>
+    <col min="5" max="5" width="10.6576576576577" style="2" customWidth="1"/>
+    <col min="6" max="6" width="19.2342342342342" style="3" customWidth="1"/>
+    <col min="7" max="7" width="41.6216216216216" style="3" customWidth="1"/>
+    <col min="8" max="16384" width="8.61261261261261" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" customHeight="1" spans="1:8">
+    <row r="1" s="1" customFormat="1" customHeight="1" spans="1:7">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1779,28 +1779,28 @@
       <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" customHeight="1" spans="1:8">
+    </row>
+    <row r="2" customHeight="1" spans="1:7">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" customHeight="1" spans="1:8">
+    <row r="3" customHeight="1" spans="1:7">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1811,16 +1811,19 @@
         <v>13</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>14</v>
       </c>
+      <c r="F3" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="G3" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" customHeight="1" spans="1:8">
+    <row r="4" customHeight="1" spans="1:7">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1831,16 +1834,19 @@
         <v>17</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>18</v>
       </c>
+      <c r="F4" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="G4" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" customHeight="1" spans="1:8">
+    <row r="5" customHeight="1" spans="1:7">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1853,11 +1859,14 @@
       <c r="E5" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="F5" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="G5" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" customHeight="1" spans="1:8">
+    <row r="6" customHeight="1" spans="1:7">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1868,16 +1877,19 @@
         <v>25</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" customHeight="1" spans="1:8">
+    <row r="7" customHeight="1" spans="1:7">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1885,16 +1897,19 @@
         <v>27</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>28</v>
       </c>
+      <c r="F7" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="G7" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="8" customHeight="1" spans="1:8">
+    <row r="8" customHeight="1" spans="1:7">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1907,11 +1922,14 @@
       <c r="E8" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="F8" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="G8" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="9" customHeight="1" spans="1:8">
+    <row r="9" customHeight="1" spans="1:7">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1921,11 +1939,14 @@
       <c r="C9" s="3" t="s">
         <v>34</v>
       </c>
+      <c r="F9" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="G9" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="10" customHeight="1" spans="1:8">
+    <row r="10" customHeight="1" spans="1:7">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1938,11 +1959,14 @@
       <c r="E10" s="2" t="s">
         <v>28</v>
       </c>
+      <c r="F10" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="G10" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="11" customHeight="1" spans="1:8">
+    <row r="11" customHeight="1" spans="1:7">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1955,11 +1979,14 @@
       <c r="E11" s="2" t="s">
         <v>41</v>
       </c>
+      <c r="F11" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="G11" s="3" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="12" customHeight="1" spans="1:8">
+    <row r="12" customHeight="1" spans="1:7">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1969,11 +1996,14 @@
       <c r="C12" s="3" t="s">
         <v>44</v>
       </c>
+      <c r="F12" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="G12" s="3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="13" customHeight="1" spans="1:8">
+    <row r="13" customHeight="1" spans="1:7">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1984,9 +2014,9 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" customHeight="1" spans="1:8">
+    <row r="14" customHeight="1" spans="1:7">
       <c r="A14" s="2">
-        <v>12</v>
+        <v>12.1</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>48</v>
@@ -1995,7 +2025,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" customHeight="1" spans="1:8">
+    <row r="15" customHeight="1" spans="1:7">
       <c r="A15" s="2">
         <v>13</v>
       </c>
@@ -2009,7 +2039,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" customHeight="1" spans="1:8">
+    <row r="16" customHeight="1" spans="1:7">
       <c r="A16" s="2">
         <v>14</v>
       </c>
@@ -2072,22 +2102,25 @@
       <c r="C20" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="D20" s="2" t="s">
         <v>66</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="21" customHeight="1" spans="1:7">
       <c r="A21" s="2">
-        <v>18</v>
+        <v>18.1</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E21" s="2" t="s">
         <v>69</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="22" customHeight="1" spans="1:7">
@@ -2095,10 +2128,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" customHeight="1" spans="1:7">
@@ -2106,10 +2139,10 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" customHeight="1" spans="1:7">
@@ -2117,10 +2150,10 @@
         <v>20.1</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="25" customHeight="1" spans="1:7">
@@ -2128,10 +2161,10 @@
         <v>21.1</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="26" customHeight="1" spans="1:7">
@@ -2139,10 +2172,10 @@
         <v>21.2</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="27" customHeight="1" spans="1:7">
@@ -2150,10 +2183,10 @@
         <v>21.3</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" customHeight="1" spans="1:7">
@@ -2161,13 +2194,13 @@
         <v>21.4</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29" customHeight="1" spans="1:7">
@@ -2175,10 +2208,10 @@
         <v>22</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" customHeight="1" spans="1:7">
@@ -2186,10 +2219,10 @@
         <v>23</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="31" customHeight="1" spans="1:7">
@@ -2197,10 +2230,10 @@
         <v>24</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="32" customHeight="1" spans="1:7">
@@ -2208,10 +2241,13 @@
         <v>25</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="33" customHeight="1" spans="1:4">
@@ -2219,10 +2255,10 @@
         <v>26</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="34" customHeight="1" spans="1:4">
@@ -2230,10 +2266,10 @@
         <v>27</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="35" customHeight="1" spans="1:4">
@@ -2241,10 +2277,10 @@
         <v>28</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36" customHeight="1" spans="1:4">
@@ -2252,13 +2288,13 @@
         <v>29</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="37" customHeight="1" spans="1:4">
@@ -2266,13 +2302,13 @@
         <v>30</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="38" customHeight="1" spans="1:4">
@@ -2280,13 +2316,13 @@
         <v>31</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="39" customHeight="1" spans="1:4">
@@ -2294,13 +2330,13 @@
         <v>32</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C39" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="40" customHeight="1" spans="1:4">
@@ -2308,10 +2344,10 @@
         <v>33</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="41" customHeight="1" spans="1:4">
@@ -2319,13 +2355,13 @@
         <v>34</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="42" customHeight="1" spans="1:4">
@@ -2333,13 +2369,13 @@
         <v>35</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="43" customHeight="1" spans="1:4">
@@ -2347,10 +2383,10 @@
         <v>36</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="44" customHeight="1" spans="1:4">
@@ -2358,10 +2394,10 @@
         <v>37</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="45" customHeight="1" spans="1:4">
@@ -2369,13 +2405,13 @@
         <v>38</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="46" customHeight="1" spans="1:4">
@@ -2383,13 +2419,13 @@
         <v>39</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="47" customHeight="1" spans="1:4">
@@ -2397,13 +2433,13 @@
         <v>40</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="48" customHeight="1" spans="1:4">
@@ -2411,231 +2447,228 @@
         <v>41</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="49" customHeight="1" spans="1:8">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="49" customHeight="1" spans="1:4">
       <c r="A49" s="2">
         <v>42</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="50" customHeight="1" spans="1:8">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="50" customHeight="1" spans="1:4">
       <c r="A50" s="2">
         <v>43</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="51" customHeight="1" spans="1:8">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="51" customHeight="1" spans="1:4">
       <c r="A51" s="2">
         <v>44</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="52" customHeight="1" spans="1:8">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="52" customHeight="1" spans="1:4">
       <c r="A52" s="2">
         <v>45</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="53" customHeight="1" spans="1:8">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="53" customHeight="1" spans="1:4">
       <c r="A53" s="2">
         <v>46</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="54" customHeight="1" spans="1:8">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="54" customHeight="1" spans="1:4">
       <c r="A54" s="2">
         <v>47</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="55" customHeight="1" spans="1:8">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="55" customHeight="1" spans="1:4">
       <c r="A55" s="2">
         <v>48</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="56" customHeight="1" spans="1:8">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="56" customHeight="1" spans="1:4">
       <c r="A56" s="2">
         <v>49</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="57" customHeight="1" spans="1:8">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="57" customHeight="1" spans="1:4">
       <c r="A57" s="2">
         <v>50</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="58" customHeight="1" spans="1:8">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="58" customHeight="1" spans="1:4">
       <c r="A58" s="2">
         <v>51</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="59" customHeight="1" spans="1:8">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="59" customHeight="1" spans="1:4">
       <c r="A59" s="2">
         <v>52</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="60" customHeight="1" spans="1:8">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="60" customHeight="1" spans="1:4">
       <c r="A60" s="2">
         <v>53</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="H60" s="6" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="61" customHeight="1" spans="1:8">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="61" customHeight="1" spans="1:4">
       <c r="A61" s="2">
         <v>54</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="62" customHeight="1" spans="1:8">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="62" customHeight="1" spans="1:4">
       <c r="A62" s="2">
         <v>55</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="63" customHeight="1" spans="1:8">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="63" customHeight="1" spans="1:4">
       <c r="A63" s="2">
         <v>55</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="64" customHeight="1" spans="1:8">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="64" customHeight="1" spans="1:4">
       <c r="A64" s="2">
         <v>56</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="65" customHeight="1" spans="1:4">
@@ -2643,10 +2676,10 @@
         <v>57</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="66" customHeight="1" spans="1:4">
@@ -2654,13 +2687,13 @@
         <v>58</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="67" customHeight="1" spans="1:4">
@@ -2668,13 +2701,13 @@
         <v>58.3</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="68" customHeight="1" spans="1:4">
@@ -2682,13 +2715,13 @@
         <v>59</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="69" customHeight="1" spans="1:4">
@@ -2696,13 +2729,13 @@
         <v>60</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="70" customHeight="1" spans="1:4">
@@ -2710,13 +2743,13 @@
         <v>61</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="71" customHeight="1" spans="1:4">
@@ -2724,22 +2757,22 @@
         <v>62</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H71" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:G71" etc:filterBottomFollowUsedRange="0">
+    <sortState ref="A2:G71">
+      <sortCondition ref="A1"/>
+    </sortState>
     <extLst/>
   </autoFilter>
-  <hyperlinks>
-    <hyperlink ref="H60" r:id="rId1" display="https://open.spotify.com/album/0AKlp3UyebGKt4o0GShbdg"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>